<commit_message>
Fix broken formula strings in How to Use sheet
Formula display strings in the instructions sheet were being stored
as live Excel formulas (starting with =). Prefixed all with a leading
space so Excel treats them as text. Also fixed a syntax error in the
LEVEL formula example (mismatched parenthesis).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PEUMhW5kWA7V6TfxKpY8jb
</commit_message>
<xml_diff>
--- a/Owner Inbox/On-Demand/CALLUM-001-BOM-ParentExtractor.xlsx
+++ b/Owner Inbox/On-Demand/CALLUM-001-BOM-ParentExtractor.xlsx
@@ -22699,9 +22699,10 @@
           <t>Add the IS_PARENT formula in column F</t>
         </is>
       </c>
-      <c r="C4" s="30">
-        <f>SUMPRODUCT(--(LEFT($A$2:$A$3000,LEN(A2)+1)=A2&amp;"."))&gt;0</f>
-        <v/>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =SUMPRODUCT(--(LEFT($A$2:$A$3000,LEN(A2)+1)=A2&amp;"."))&gt;0</t>
+        </is>
       </c>
       <c r="D4" s="30" t="inlineStr">
         <is>
@@ -22720,13 +22721,14 @@
           <t>Add the LEVEL formula in column G</t>
         </is>
       </c>
-      <c r="C5" s="28">
-        <f>LEN(A2)-LEN(SUBSTITUTE(A2,".",""))+1</f>
-        <v/>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =LEN(A2)-LEN(SUBSTITUTE(A2,".",""))+1</t>
+        </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>Counts dots in ITEM NO. and adds 1. Item '1.2.3' = 3 dots + 1 = level 4. Wait — 2 dots = level 3. Formula is correct.</t>
+          <t>Counts dots in ITEM NO. and adds 1. Item '1.2.3' has 2 dots → level 3.</t>
         </is>
       </c>
     </row>
@@ -22810,9 +22812,10 @@
           <t>IS_PARENT (Col F)</t>
         </is>
       </c>
-      <c r="B11" s="33">
-        <f>SUMPRODUCT(--(LEFT($A$2:$A$3000,LEN(A2)+1)=A2&amp;"."))&gt;0</f>
-        <v/>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =SUMPRODUCT(--(LEFT($A$2:$A$3000,LEN(A2)+1)=A2&amp;"."))&gt;0</t>
+        </is>
       </c>
       <c r="C11" s="34" t="inlineStr">
         <is>
@@ -22831,13 +22834,14 @@
           <t>LEVEL (Col G)</t>
         </is>
       </c>
-      <c r="B12" s="36">
-        <f>LEN(A2)-LEN(SUBSTITUTE(A2,".","")+1</f>
-        <v/>
+      <c r="B12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =LEN(A2)-LEN(SUBSTITUTE(A2,".",""  ))+1</t>
+        </is>
       </c>
       <c r="C12" s="37" t="inlineStr">
         <is>
-          <t>Counts hierarchy depth from dot count in ITEM NO.</t>
+          <t>Counts hierarchy depth from dot count in ITEM NO. '1.2.3' → 2 dots + 1 = level 3.</t>
         </is>
       </c>
       <c r="D12" s="37" t="inlineStr"/>
@@ -22848,13 +22852,14 @@
           <t>DIRECT CHILD COUNT</t>
         </is>
       </c>
-      <c r="B13" s="33">
-        <f>SUMPRODUCT((LEFT($A$2:$A$3000,LEN(A2)+1)=A2&amp;".")*(LEN($A$2:$A$3000)-LEN(SUBSTITUTE($A$2:$A$3000,".","")))=LEN(A2)-LEN(SUBSTITUTE(A2,".",""))+1)</f>
-        <v/>
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =COUNTIF($A$2:$A$3000,A2&amp;".*")-COUNTIF($A$2:$A$3000,A2&amp;".*.*")</t>
+        </is>
       </c>
       <c r="C13" s="34" t="inlineStr">
         <is>
-          <t>Counts immediate children only (not grandchildren)</t>
+          <t>Counts direct children only (not grandchildren).</t>
         </is>
       </c>
       <c r="D13" s="34" t="inlineStr">

</xml_diff>